<commit_message>
Updated and fully working till tasks
</commit_message>
<xml_diff>
--- a/CRMLeaf PSA.xlsx
+++ b/CRMLeaf PSA.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R20"/>
+  <dimension ref="A1:R26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2174,6 +2174,534 @@
         <v>1</v>
       </c>
       <c r="R20" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>PSA-0020</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>08c40dbe19e6880a0fd094ca674c47b3</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>RUN_20260929_111603</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>PSA</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Project Creation</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>ScriptError</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>ScriptError in Project Creation</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>1. Authenticate to CRMLeaf.
+2. Execute Project Creation workflow sequence.</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>Module Project Creation passes all UI invariants without blocking.</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>Locator.click: Timeout 30000ms exceeded.</t>
+        </is>
+      </c>
+      <c r="L21">
+        <f>HYPERLINK("evidence_output\RUN_20260929_111603\Project_Creation.png", "Screenshot")</f>
+        <v/>
+      </c>
+      <c r="M21">
+        <f>HYPERLINK("evidence\RUN_20260929_111603\Project_Creation\video\page@990eb22767e08c753cf707967afc31c5.webm", "Video")</f>
+        <v/>
+      </c>
+      <c r="N21">
+        <f>HYPERLINK("evidence_output\RUN_20260929_111603\Project_Creation_diagnostics.log", "Logs")</f>
+        <v/>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>2026-09-29 11:18:50</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>2026-09-29 11:18:50</t>
+        </is>
+      </c>
+      <c r="Q21" t="n">
+        <v>1</v>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>PSA-0021</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>cf63e74cb43d85a4e1aacf1aaee752da</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>RUN_20260929_112058</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>PSA</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Project Overview</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>ScriptError</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>ScriptError in Project Overview</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>1. Authenticate to CRMLeaf.
+2. Execute Project Overview workflow sequence.</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Module Project Overview passes all UI invariants without blocking.</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>Locator.wait_for: Timeout 10000ms exceeded.</t>
+        </is>
+      </c>
+      <c r="L22">
+        <f>HYPERLINK("evidence_output\RUN_20260929_112058\Project_Overview.png", "Screenshot")</f>
+        <v/>
+      </c>
+      <c r="M22">
+        <f>HYPERLINK("evidence\RUN_20260929_112058\Project_Overview\video\page@4b5c893d91000b38154d963cb3b520e5.webm", "Video")</f>
+        <v/>
+      </c>
+      <c r="N22">
+        <f>HYPERLINK("evidence_output\RUN_20260929_112058\Project_Overview_diagnostics.log", "Logs")</f>
+        <v/>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>2026-09-29 11:23:44</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>2026-09-29 12:49:47</t>
+        </is>
+      </c>
+      <c r="Q22" t="n">
+        <v>5</v>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>Reproduced</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>PSA-0022</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>e10c92b766f5d51f51910168ac4edbde</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>RUN_20260929_121429</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>PSA</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Project Overview</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>ScriptError</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>ScriptError in Project Overview</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>1. Authenticate to CRMLeaf.
+2. Execute Project Overview workflow sequence.</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Module Project Overview passes all UI invariants without blocking.</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>Locator.click: Timeout 30000ms exceeded.</t>
+        </is>
+      </c>
+      <c r="L23">
+        <f>HYPERLINK("evidence_output\RUN_20260929_121429\Project_Overview.png", "Screenshot")</f>
+        <v/>
+      </c>
+      <c r="M23">
+        <f>HYPERLINK("evidence\RUN_20260929_121429\Project_Overview\video\page@6f4288d232102d262a73791f936e4c2c.webm", "Video")</f>
+        <v/>
+      </c>
+      <c r="N23">
+        <f>HYPERLINK("evidence_output\RUN_20260929_121429\Project_Overview_diagnostics.log", "Logs")</f>
+        <v/>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>2026-09-29 12:18:02</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>2026-09-29 12:18:02</t>
+        </is>
+      </c>
+      <c r="Q23" t="n">
+        <v>1</v>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>PSA-0023</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>be60a847e3b712ca130729782f57e88b</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>RUN_20260929_123019</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>PSA</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Project Creation</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>ProductDefect</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>ProductDefect in Project Creation</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>1. Authenticate to CRMLeaf.
+2. Execute Project Creation workflow sequence.</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Module Project Creation passes all UI invariants without blocking.</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>name 'cite' is not defined</t>
+        </is>
+      </c>
+      <c r="L24">
+        <f>HYPERLINK("evidence_output\RUN_20260929_123019\Project_Creation.png", "Screenshot")</f>
+        <v/>
+      </c>
+      <c r="M24">
+        <f>HYPERLINK("evidence\RUN_20260929_123019\Project_Creation\video\page@568721f1955b9da7dba5c4b44438141b.webm", "Video")</f>
+        <v/>
+      </c>
+      <c r="N24">
+        <f>HYPERLINK("evidence_output\RUN_20260929_123019\Project_Creation_diagnostics.log", "Logs")</f>
+        <v/>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>2026-09-29 12:32:32</t>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>2026-09-29 12:36:21</t>
+        </is>
+      </c>
+      <c r="Q24" t="n">
+        <v>2</v>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>Reproduced</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>PSA-0024</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>052e090c92469a2a7a6e1a1b5fe3e63a</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>RUN_20260929_125113</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>PSA</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Project Creation</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>ProductDefect</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>ProductDefect in Project Creation</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>1. Authenticate to CRMLeaf.
+2. Execute Project Creation workflow sequence.</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>Module Project Creation passes all UI invariants without blocking.</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>Project save failed: Form did not close. Check for validation errors (e.g., missing mandatory fields).</t>
+        </is>
+      </c>
+      <c r="L25">
+        <f>HYPERLINK("evidence_output\RUN_20260929_125113\Project_Creation.png", "Screenshot")</f>
+        <v/>
+      </c>
+      <c r="M25">
+        <f>HYPERLINK("evidence\RUN_20260929_125113\Project_Creation\video\page@fba37c2616de55bf151c561aac15e5f3.webm", "Video")</f>
+        <v/>
+      </c>
+      <c r="N25">
+        <f>HYPERLINK("evidence_output\RUN_20260929_125113\Project_Creation_diagnostics.log", "Logs")</f>
+        <v/>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>2026-09-29 12:53:49</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>2026-09-29 12:53:49</t>
+        </is>
+      </c>
+      <c r="Q25" t="n">
+        <v>1</v>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>PSA-0025</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>5bc3737ba29c1766da573763c0181d18</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>RUN_20260929_125519</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>PSA</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Project Creation</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>ProductDefect</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>ProductDefect in Project Creation</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>1. Authenticate to CRMLeaf.
+2. Execute Project Creation workflow sequence.</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>Module Project Creation passes all UI invariants without blocking.</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>Page.goto: net::ERR_ABORTED at https://www.crmleaf.com/account/projects</t>
+        </is>
+      </c>
+      <c r="L26">
+        <f>HYPERLINK("evidence_output\RUN_20260929_125519\Project_Creation.png", "Screenshot")</f>
+        <v/>
+      </c>
+      <c r="M26">
+        <f>HYPERLINK("evidence\RUN_20260929_125519\Project_Creation\video\page@e83583dedea78ea41a96553263cf60cd.webm", "Video")</f>
+        <v/>
+      </c>
+      <c r="N26">
+        <f>HYPERLINK("evidence_output\RUN_20260929_125519\Project_Creation_diagnostics.log", "Logs")</f>
+        <v/>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>2026-09-29 12:57:50</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>2026-09-29 12:57:50</t>
+        </is>
+      </c>
+      <c r="Q26" t="n">
+        <v>1</v>
+      </c>
+      <c r="R26" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
@@ -2190,7 +2718,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:G22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2488,6 +3016,354 @@
       <c r="G10" t="inlineStr">
         <is>
           <t>FAILED</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>RUN_20260929_111603</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2026-09-29 11:18:50</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>11</v>
+      </c>
+      <c r="D11" t="n">
+        <v>7</v>
+      </c>
+      <c r="E11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" t="n">
+        <v>3</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>RUN_20260929_112058</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2026-09-29 11:23:44</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>11</v>
+      </c>
+      <c r="D12" t="n">
+        <v>8</v>
+      </c>
+      <c r="E12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" t="n">
+        <v>2</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>RUN_20260929_121007</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2026-09-29 12:12:58</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>11</v>
+      </c>
+      <c r="D13" t="n">
+        <v>8</v>
+      </c>
+      <c r="E13" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" t="n">
+        <v>2</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>RUN_20260929_121429</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2026-09-29 12:18:02</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>11</v>
+      </c>
+      <c r="D14" t="n">
+        <v>8</v>
+      </c>
+      <c r="E14" t="n">
+        <v>1</v>
+      </c>
+      <c r="F14" t="n">
+        <v>2</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>RUN_20260929_121938</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>2026-09-29 12:22:39</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>11</v>
+      </c>
+      <c r="D15" t="n">
+        <v>8</v>
+      </c>
+      <c r="E15" t="n">
+        <v>1</v>
+      </c>
+      <c r="F15" t="n">
+        <v>2</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>RUN_20260929_123019</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>2026-09-29 12:32:33</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>11</v>
+      </c>
+      <c r="D16" t="n">
+        <v>7</v>
+      </c>
+      <c r="E16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F16" t="n">
+        <v>3</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>RUN_20260929_123345</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>2026-09-29 12:36:21</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>11</v>
+      </c>
+      <c r="D17" t="n">
+        <v>7</v>
+      </c>
+      <c r="E17" t="n">
+        <v>1</v>
+      </c>
+      <c r="F17" t="n">
+        <v>3</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>RUN_20260929_123758</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>2026-09-29 12:41:27</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>11</v>
+      </c>
+      <c r="D18" t="n">
+        <v>8</v>
+      </c>
+      <c r="E18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F18" t="n">
+        <v>2</v>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>RUN_20260929_124631</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>2026-09-29 12:49:47</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>11</v>
+      </c>
+      <c r="D19" t="n">
+        <v>8</v>
+      </c>
+      <c r="E19" t="n">
+        <v>1</v>
+      </c>
+      <c r="F19" t="n">
+        <v>2</v>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>RUN_20260929_125113</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>2026-09-29 12:53:49</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>11</v>
+      </c>
+      <c r="D20" t="n">
+        <v>7</v>
+      </c>
+      <c r="E20" t="n">
+        <v>1</v>
+      </c>
+      <c r="F20" t="n">
+        <v>3</v>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>RUN_20260929_125519</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>2026-09-29 12:57:50</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>11</v>
+      </c>
+      <c r="D21" t="n">
+        <v>7</v>
+      </c>
+      <c r="E21" t="n">
+        <v>1</v>
+      </c>
+      <c r="F21" t="n">
+        <v>3</v>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>RUN_20260929_125936</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>2026-09-29 13:03:06</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>11</v>
+      </c>
+      <c r="D22" t="n">
+        <v>11</v>
+      </c>
+      <c r="E22" t="n">
+        <v>0</v>
+      </c>
+      <c r="F22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Updated and fully working without budget
</commit_message>
<xml_diff>
--- a/CRMLeaf PSA.xlsx
+++ b/CRMLeaf PSA.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R26"/>
+  <dimension ref="A1:R34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2255,15 +2255,15 @@
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>2026-09-29 11:18:50</t>
+          <t>2026-09-29 14:02:44</t>
         </is>
       </c>
       <c r="Q21" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>Draft</t>
+          <t>Reproduced</t>
         </is>
       </c>
     </row>
@@ -2343,11 +2343,11 @@
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>2026-09-29 12:49:47</t>
+          <t>2026-09-29 16:13:10</t>
         </is>
       </c>
       <c r="Q22" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="R22" t="inlineStr">
         <is>
@@ -2704,6 +2704,710 @@
       <c r="R26" t="inlineStr">
         <is>
           <t>Draft</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>PSA-0026</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>73949667ecde0696de5d48b56bd85f12</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>RUN_20260929_135345</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>PSA</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Tasks</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>ScriptError</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>ScriptError in Tasks</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>1. Authenticate to CRMLeaf.
+2. Execute Tasks workflow sequence.</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>Module Tasks passes all UI invariants without blocking.</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>Locator.wait_for: Timeout 5000ms exceeded.</t>
+        </is>
+      </c>
+      <c r="L27">
+        <f>HYPERLINK("evidence_output\RUN_20260929_135345\Tasks.png", "Screenshot")</f>
+        <v/>
+      </c>
+      <c r="M27">
+        <f>HYPERLINK("evidence\RUN_20260929_135345\Tasks\video\page@179187cf92e8013cf87973d37b5dd774.webm", "Video")</f>
+        <v/>
+      </c>
+      <c r="N27">
+        <f>HYPERLINK("evidence_output\RUN_20260929_135345\Tasks_diagnostics.log", "Logs")</f>
+        <v/>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>2026-09-29 13:57:08</t>
+        </is>
+      </c>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>2026-09-29 13:57:08</t>
+        </is>
+      </c>
+      <c r="Q27" t="n">
+        <v>1</v>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>PSA-0027</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>a03c6d0d32fb89cc5720dffd542b5fdd</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>RUN_20260929_135345</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>PSA</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Invoices</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>ScriptError</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>ScriptError in Invoices</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>1. Authenticate to CRMLeaf.
+2. Execute Invoices workflow sequence.</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>Module Invoices passes all UI invariants without blocking.</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>Locator.wait_for: Timeout 15000ms exceeded.</t>
+        </is>
+      </c>
+      <c r="L28">
+        <f>HYPERLINK("evidence_output\RUN_20260929_135345\Invoices.png", "Screenshot")</f>
+        <v/>
+      </c>
+      <c r="M28">
+        <f>HYPERLINK("evidence\RUN_20260929_135345\Invoices\video\page@7382fb7bb17ae4fd3c8b44e63a821405.webm", "Video")</f>
+        <v/>
+      </c>
+      <c r="N28">
+        <f>HYPERLINK("evidence_output\RUN_20260929_135345\Invoices_diagnostics.log", "Logs")</f>
+        <v/>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>2026-09-29 13:57:50</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>2026-09-29 14:23:39</t>
+        </is>
+      </c>
+      <c r="Q28" t="n">
+        <v>2</v>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>Reproduced</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>PSA-0028</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>470b7955cc8718987336282b758e6640</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>RUN_20260929_141907</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>PSA</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Time Sheet</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>ProductDefect</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>ProductDefect in Time Sheet</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>1. Authenticate to CRMLeaf.
+2. Execute Time Sheet workflow sequence.</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>Module Time Sheet passes all UI invariants without blocking.</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>Locator.is_visible: Unexpected token "=" while parsing css selector "table tbody tr, text='Automated Timesheet Verification'". Did you mean to CSS.escape it?</t>
+        </is>
+      </c>
+      <c r="L29">
+        <f>HYPERLINK("evidence_output\RUN_20260929_141907\Time_Sheet.png", "Screenshot")</f>
+        <v/>
+      </c>
+      <c r="M29">
+        <f>HYPERLINK("evidence\RUN_20260929_141907\Time_Sheet\video\page@18c2bad1478c2c7cd5f2519a384f3dcd.webm", "Video")</f>
+        <v/>
+      </c>
+      <c r="N29">
+        <f>HYPERLINK("evidence_output\RUN_20260929_141907\Time_Sheet_diagnostics.log", "Logs")</f>
+        <v/>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>2026-09-29 14:22:51</t>
+        </is>
+      </c>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>2026-09-29 14:54:37</t>
+        </is>
+      </c>
+      <c r="Q29" t="n">
+        <v>2</v>
+      </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>Reproduced</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>PSA-0029</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>6103844c37da224cd99c31bf16d9113e</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>RUN_20260929_142730</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>PSA</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Lead Creation</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>ProductDefect</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>ProductDefect in Lead Creation</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>1. Authenticate to CRMLeaf.
+2. Execute Lead Creation workflow sequence.</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>Module Lead Creation passes all UI invariants without blocking.</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>Lead creation failed validation: The Deal Name field is required.</t>
+        </is>
+      </c>
+      <c r="L30">
+        <f>HYPERLINK("evidence_output\RUN_20260929_142730\Lead_Creation.png", "Screenshot")</f>
+        <v/>
+      </c>
+      <c r="M30">
+        <f>HYPERLINK("evidence\RUN_20260929_142730\Lead_Creation\video\page@9fffcd6208d4786e2f2e9c2ceb85e6ae.webm", "Video")</f>
+        <v/>
+      </c>
+      <c r="N30">
+        <f>HYPERLINK("evidence_output\RUN_20260929_142730\Lead_Creation_diagnostics.log", "Logs")</f>
+        <v/>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>2026-09-29 14:28:20</t>
+        </is>
+      </c>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>2026-09-29 14:28:20</t>
+        </is>
+      </c>
+      <c r="Q30" t="n">
+        <v>1</v>
+      </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>PSA-0030</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>4af7d1fe720c2c9d96471ec67a77c819</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>RUN_20260929_142932</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>PSA</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Lead Creation</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>ProductDefect</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>ProductDefect in Lead Creation</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>1. Authenticate to CRMLeaf.
+2. Execute Lead Creation workflow sequence.</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>Module Lead Creation passes all UI invariants without blocking.</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>Lead creation failed validation: Please select a company from the dropdown.</t>
+        </is>
+      </c>
+      <c r="L31">
+        <f>HYPERLINK("evidence_output\RUN_20260929_142932\Lead_Creation.png", "Screenshot")</f>
+        <v/>
+      </c>
+      <c r="M31">
+        <f>HYPERLINK("evidence\RUN_20260929_142932\Lead_Creation\video\page@927b224cbf005582d6cedc91f50795f7.webm", "Video")</f>
+        <v/>
+      </c>
+      <c r="N31">
+        <f>HYPERLINK("evidence_output\RUN_20260929_142932\Lead_Creation_diagnostics.log", "Logs")</f>
+        <v/>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>2026-09-29 14:30:21</t>
+        </is>
+      </c>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>2026-09-29 16:00:33</t>
+        </is>
+      </c>
+      <c r="Q31" t="n">
+        <v>8</v>
+      </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>Reproduced</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>PSA-0031</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>1853d489ec35c12e09ce72a6711b2492</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>RUN_20260929_145038</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>PSA</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Payment</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>ScriptError</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>ScriptError in Payment</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>1. Authenticate to CRMLeaf.
+2. Execute Payment workflow sequence.</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>Module Payment passes all UI invariants without blocking.</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>Locator.scroll_into_view_if_needed: Timeout 30000ms exceeded.</t>
+        </is>
+      </c>
+      <c r="L32">
+        <f>HYPERLINK("evidence_output\RUN_20260929_145038\Payment.png", "Screenshot")</f>
+        <v/>
+      </c>
+      <c r="M32">
+        <f>HYPERLINK("evidence\RUN_20260929_145038\Payment\video\page@4e7a3872b9ba6c5020e5bb96949305b3.webm", "Video")</f>
+        <v/>
+      </c>
+      <c r="N32">
+        <f>HYPERLINK("evidence_output\RUN_20260929_145038\Payment_diagnostics.log", "Logs")</f>
+        <v/>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>2026-09-29 14:56:00</t>
+        </is>
+      </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>2026-09-29 14:56:00</t>
+        </is>
+      </c>
+      <c r="Q32" t="n">
+        <v>1</v>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>PSA-0032</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>014009dbf0b4b909661a8d9c5af1331b</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>RUN_20260929_154413</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>PSA</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Lead Creation</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>ProductDefect</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>ProductDefect in Lead Creation</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>1. Authenticate to CRMLeaf.
+2. Execute Lead Creation workflow sequence.</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>Module Lead Creation passes all UI invariants without blocking.</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>Lead creation failed validation: Form did not submit</t>
+        </is>
+      </c>
+      <c r="L33">
+        <f>HYPERLINK("evidence_output\RUN_20260929_154413\Lead_Creation.png", "Screenshot")</f>
+        <v/>
+      </c>
+      <c r="M33">
+        <f>HYPERLINK("evidence\RUN_20260929_154413\Lead_Creation\video\page@783c5fd21a8200008dbbef30d099785c.webm", "Video")</f>
+        <v/>
+      </c>
+      <c r="N33">
+        <f>HYPERLINK("evidence_output\RUN_20260929_154413\Lead_Creation_diagnostics.log", "Logs")</f>
+        <v/>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>2026-09-29 15:45:00</t>
+        </is>
+      </c>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>2026-09-29 15:45:00</t>
+        </is>
+      </c>
+      <c r="Q33" t="n">
+        <v>1</v>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>PSA-0033</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>7556e15c768d4d0c75ff0a6ccb1e4dfa</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>RUN_20260929_160439</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>PSA</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Proposal Acceptance</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>ScriptError</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>ScriptError in Proposal Acceptance</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>1. Authenticate to CRMLeaf.
+2. Execute Proposal Acceptance workflow sequence.</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>Module Proposal Acceptance passes all UI invariants without blocking.</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>Locator.click: Timeout 30000ms exceeded.</t>
+        </is>
+      </c>
+      <c r="L34">
+        <f>HYPERLINK("evidence_output\RUN_20260929_160439\Proposal_Acceptance.png", "Screenshot")</f>
+        <v/>
+      </c>
+      <c r="M34">
+        <f>HYPERLINK("evidence\RUN_20260929_160439\Proposal_Acceptance\video\page@e8f4c6080c9a047402339d8a2adfa572.webm", "Video")</f>
+        <v/>
+      </c>
+      <c r="N34">
+        <f>HYPERLINK("evidence_output\RUN_20260929_160439\Proposal_Acceptance_diagnostics.log", "Logs")</f>
+        <v/>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>2026-09-29 16:06:41</t>
+        </is>
+      </c>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>2026-09-29 16:11:47</t>
+        </is>
+      </c>
+      <c r="Q34" t="n">
+        <v>2</v>
+      </c>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>Reproduced</t>
         </is>
       </c>
     </row>
@@ -2718,7 +3422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G22"/>
+  <dimension ref="A1:G42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3362,6 +4066,586 @@
         <v>0</v>
       </c>
       <c r="G22" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>RUN_20260929_135345</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>2026-09-29 13:57:50</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>17</v>
+      </c>
+      <c r="D23" t="n">
+        <v>11</v>
+      </c>
+      <c r="E23" t="n">
+        <v>2</v>
+      </c>
+      <c r="F23" t="n">
+        <v>4</v>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>RUN_20260929_135953</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>2026-09-29 14:02:44</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>17</v>
+      </c>
+      <c r="D24" t="n">
+        <v>7</v>
+      </c>
+      <c r="E24" t="n">
+        <v>1</v>
+      </c>
+      <c r="F24" t="n">
+        <v>9</v>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>RUN_20260929_140514</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>2026-09-29 14:08:13</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>17</v>
+      </c>
+      <c r="D25" t="n">
+        <v>8</v>
+      </c>
+      <c r="E25" t="n">
+        <v>1</v>
+      </c>
+      <c r="F25" t="n">
+        <v>8</v>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>RUN_20260929_141423</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>2026-09-29 14:17:25</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>17</v>
+      </c>
+      <c r="D26" t="n">
+        <v>8</v>
+      </c>
+      <c r="E26" t="n">
+        <v>1</v>
+      </c>
+      <c r="F26" t="n">
+        <v>8</v>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>RUN_20260929_141907</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>2026-09-29 14:23:40</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>17</v>
+      </c>
+      <c r="D27" t="n">
+        <v>14</v>
+      </c>
+      <c r="E27" t="n">
+        <v>2</v>
+      </c>
+      <c r="F27" t="n">
+        <v>1</v>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>RUN_20260929_142730</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>2026-09-29 14:28:20</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>17</v>
+      </c>
+      <c r="D28" t="n">
+        <v>0</v>
+      </c>
+      <c r="E28" t="n">
+        <v>1</v>
+      </c>
+      <c r="F28" t="n">
+        <v>16</v>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>RUN_20260929_142932</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>2026-09-29 14:30:22</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>17</v>
+      </c>
+      <c r="D29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E29" t="n">
+        <v>1</v>
+      </c>
+      <c r="F29" t="n">
+        <v>16</v>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>RUN_20260929_143132</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>2026-09-29 14:32:11</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>17</v>
+      </c>
+      <c r="D30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E30" t="n">
+        <v>1</v>
+      </c>
+      <c r="F30" t="n">
+        <v>16</v>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>RUN_20260929_143506</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>2026-09-29 14:35:51</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>17</v>
+      </c>
+      <c r="D31" t="n">
+        <v>0</v>
+      </c>
+      <c r="E31" t="n">
+        <v>1</v>
+      </c>
+      <c r="F31" t="n">
+        <v>16</v>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>RUN_20260929_144446</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>2026-09-29 14:45:35</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>17</v>
+      </c>
+      <c r="D32" t="n">
+        <v>0</v>
+      </c>
+      <c r="E32" t="n">
+        <v>1</v>
+      </c>
+      <c r="F32" t="n">
+        <v>16</v>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>RUN_20260929_145038</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>2026-09-29 14:56:00</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>17</v>
+      </c>
+      <c r="D33" t="n">
+        <v>15</v>
+      </c>
+      <c r="E33" t="n">
+        <v>2</v>
+      </c>
+      <c r="F33" t="n">
+        <v>0</v>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>RUN_20260929_151316</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>2026-09-29 15:18:31</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>17</v>
+      </c>
+      <c r="D34" t="n">
+        <v>17</v>
+      </c>
+      <c r="E34" t="n">
+        <v>0</v>
+      </c>
+      <c r="F34" t="n">
+        <v>0</v>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>RUN_20260929_154413</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>2026-09-29 15:45:00</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>17</v>
+      </c>
+      <c r="D35" t="n">
+        <v>0</v>
+      </c>
+      <c r="E35" t="n">
+        <v>1</v>
+      </c>
+      <c r="F35" t="n">
+        <v>16</v>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>RUN_20260929_154746</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>2026-09-29 15:48:31</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>17</v>
+      </c>
+      <c r="D36" t="n">
+        <v>0</v>
+      </c>
+      <c r="E36" t="n">
+        <v>1</v>
+      </c>
+      <c r="F36" t="n">
+        <v>16</v>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>RUN_20260929_155551</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>2026-09-29 15:56:52</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>17</v>
+      </c>
+      <c r="D37" t="n">
+        <v>0</v>
+      </c>
+      <c r="E37" t="n">
+        <v>1</v>
+      </c>
+      <c r="F37" t="n">
+        <v>16</v>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>RUN_20260929_155738</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>2026-09-29 15:58:31</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>17</v>
+      </c>
+      <c r="D38" t="n">
+        <v>0</v>
+      </c>
+      <c r="E38" t="n">
+        <v>1</v>
+      </c>
+      <c r="F38" t="n">
+        <v>16</v>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>RUN_20260929_155947</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>2026-09-29 16:00:34</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>17</v>
+      </c>
+      <c r="D39" t="n">
+        <v>0</v>
+      </c>
+      <c r="E39" t="n">
+        <v>1</v>
+      </c>
+      <c r="F39" t="n">
+        <v>16</v>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>RUN_20260929_160439</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>2026-09-29 16:08:08</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>17</v>
+      </c>
+      <c r="D40" t="n">
+        <v>6</v>
+      </c>
+      <c r="E40" t="n">
+        <v>2</v>
+      </c>
+      <c r="F40" t="n">
+        <v>9</v>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>RUN_20260929_160947</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>2026-09-29 16:13:10</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>17</v>
+      </c>
+      <c r="D41" t="n">
+        <v>6</v>
+      </c>
+      <c r="E41" t="n">
+        <v>2</v>
+      </c>
+      <c r="F41" t="n">
+        <v>9</v>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>RUN_20260929_162619</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>2026-09-29 16:31:32</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>17</v>
+      </c>
+      <c r="D42" t="n">
+        <v>17</v>
+      </c>
+      <c r="E42" t="n">
+        <v>0</v>
+      </c>
+      <c r="F42" t="n">
+        <v>0</v>
+      </c>
+      <c r="G42" t="inlineStr">
         <is>
           <t>PASSED</t>
         </is>

</xml_diff>

<commit_message>
Updated and fully working but budget not working
</commit_message>
<xml_diff>
--- a/CRMLeaf PSA.xlsx
+++ b/CRMLeaf PSA.xlsx
@@ -3311,15 +3311,15 @@
       </c>
       <c r="P33" t="inlineStr">
         <is>
-          <t>2026-09-29 15:45:00</t>
+          <t>2026-09-29 16:45:04</t>
         </is>
       </c>
       <c r="Q33" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R33" t="inlineStr">
         <is>
-          <t>Draft</t>
+          <t>Reproduced</t>
         </is>
       </c>
     </row>
@@ -3422,7 +3422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G42"/>
+  <dimension ref="A1:G43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4648,6 +4648,35 @@
       <c r="G42" t="inlineStr">
         <is>
           <t>PASSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>RUN_20260929_164416</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>2026-09-29 16:45:04</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>18</v>
+      </c>
+      <c r="D43" t="n">
+        <v>0</v>
+      </c>
+      <c r="E43" t="n">
+        <v>1</v>
+      </c>
+      <c r="F43" t="n">
+        <v>17</v>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>FAILED</t>
         </is>
       </c>
     </row>

</xml_diff>